<commit_message>
Changing some test forms...
</commit_message>
<xml_diff>
--- a/test/sample_forms/Form-1DI - interim.xlsx
+++ b/test/sample_forms/Form-1DI - interim.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\dev\git\BitBucket workspaces\IOTC-ws\R libs\workflow\test_forms\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\dev\git\BitBucket workspaces\IOTC-ws\R libs\base\forms\base-form-management\test\sample_forms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D54F421-7A10-4D43-9E8A-3AFD3DA0F57A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD7B9087-71D8-4292-BFA7-87913F284F70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Z3raniWjLRXszYCbzXa/TU1R8wd1kHrHNccmNn7mHkAZRDJmvrP7BMraCIbrDBSr6tBMzuhQ6TxYUg6cyC/1Bg==" workbookSaltValue="C01nC0I7gdRYfsDcA3RybQ==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30120" yWindow="2700" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="93">
   <si>
     <t>Focal point</t>
   </si>
@@ -310,6 +310,12 @@
   </si>
   <si>
     <t>1.0.0-interim</t>
+  </si>
+  <si>
+    <t>FOO</t>
+  </si>
+  <si>
+    <t>SNAFU</t>
   </si>
 </sst>
 </file>
@@ -3129,7 +3135,7 @@
         <v>79</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="68"/>
@@ -3494,7 +3500,7 @@
         <v>80</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="E16" s="33" t="s">
         <v>42</v>
@@ -3862,9 +3868,7 @@
       <c r="C19" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="33" t="s">
-        <v>82</v>
-      </c>
+      <c r="D19" s="33"/>
       <c r="E19" s="33" t="s">
         <v>42</v>
       </c>

</xml_diff>